<commit_message>
Phase 105: fix MEGA TEST 4 and the three CI-only failures
- Re-export ALG-01..ALG-20: ALG-20 cited objectives.py and
  conclusion_tables.py line numbers from before Phase 101 edited them
  (T105.4 caught it). Thesis pack rebuilt from the fresh export.
- Thesis copy check hashes SVG newline-normalized, like the other text
  suffixes: CI checks out LF, the manifest was digested from CRLF.
- The completeness checks excuse an item only when its missing file is
  gitignored (FE-03 parquet), per the standing skip-not-fail rule.

MEGA TEST 4 now 115/115 locally with --runslow; CI simulated with the
feature matrix hidden: passed/skipped, no failures.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/00_evidence_index/evidence_index.xlsx
+++ b/outputs/00_evidence_index/evidence_index.xlsx
@@ -9795,12 +9795,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ALG-01</t>
+          <t>T01</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>O1, O6</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -9808,27 +9808,27 @@
       <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Dataset loading and master metadata construction</t>
+          <t>Dataset Inventory</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.txt</t>
+          <t>outputs/01_dataset_audit/T01_dataset_inventory.csv</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>src/data_loader/catalog.py; src/data_loader/circor.py; src/data_loader/duplicates.py; src/data_loader/integrity.py; src/data_loader/master.py; src/data_loader/pascal.py; src/data_loader/physionet.py</t>
+          <t>outputs/01_dataset_audit/dataset_inventory.csv</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-01</t>
+          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:08.127289+00:00</t>
+          <t>2026-08-30T10:47:59.290988+00:00</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -9838,19 +9838,19 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>file and 7 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ALG-02</t>
+          <t>T02</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
@@ -9858,27 +9858,27 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Signal harmonization and resampling</t>
+          <t>Class Distribution and Imbalance Ratio</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.txt</t>
+          <t>outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.csv</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>src/preprocessing/io.py; src/preprocessing/pipeline.py; src/preprocessing/quality.py</t>
+          <t>outputs/01_dataset_audit/class_distribution.csv</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-02</t>
+          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:08.264133+00:00</t>
+          <t>2026-08-30T10:48:00.613926+00:00</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -9888,19 +9888,19 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ALG-03</t>
+          <t>T03</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -9908,27 +9908,27 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Butterworth filtering and z-score normalization</t>
+          <t>Recording Duration and Sampling Summary</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.txt</t>
+          <t>outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.csv</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>src/preprocessing/filters.py; src/preprocessing/normalize.py</t>
+          <t>outputs/01_dataset_audit/recording_duration_summary.csv; outputs/01_dataset_audit/sampling_rate_summary.csv</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-03</t>
+          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:10.698368+00:00</t>
+          <t>2026-08-30T10:48:01.979486+00:00</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -9945,12 +9945,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ALG-04</t>
+          <t>T04</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O3 (preprocessing pipeline)</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
@@ -9958,27 +9958,27 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Multi-domain 138-feature extraction</t>
+          <t>Preprocessing Configuration</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt</t>
+          <t>outputs/02_preprocessing/T04_preprocessing_configuration.csv</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>src/feature_extraction/extractor.py; src/feature_extraction/registry.py</t>
+          <t>outputs/02_preprocessing/preprocessing_settings.csv</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-04</t>
+          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:10.830218+00:00</t>
+          <t>2026-08-30T10:48:03.098584+00:00</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -9988,19 +9988,19 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ALG-05</t>
+          <t>T05</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -10008,27 +10008,27 @@
       <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Fold-safe scaling and preprocessing</t>
+          <t>Feature Inventory and Counts</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.txt</t>
+          <t>outputs/03_features/T05_feature_inventory_and_counts.csv</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>src/data_loader/splits.py; src/models/pipeline.py</t>
+          <t>outputs/03_features/feature_inventory.csv; outputs/03_features/feature_family_summary.csv</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-05</t>
+          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:10.951681+00:00</t>
+          <t>2026-08-30T10:48:04.059902+00:00</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -10045,12 +10045,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>ALG-06</t>
+          <t>T06</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>O5</t>
+          <t>O5 (model configuration)</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -10058,27 +10058,27 @@
       <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Search based feature selection</t>
+          <t>Model Hyperparameter Configuration</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-06_search_based_feature_selection.txt</t>
+          <t>outputs/04_models/T06_model_hyperparameter_configuration.csv</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>src/feature_selection/ranking.py; src/feature_selection/sweep.py; src/optimization/base.py; src/optimization/multi_objective.py</t>
+          <t>outputs/04_models/model_registry.csv; outputs/04_models/model_search_spaces.csv</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-06</t>
+          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:11.118184+00:00</t>
+          <t>2026-08-30T10:48:05.360215+00:00</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -10088,19 +10088,19 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ALG-07</t>
+          <t>G01</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>O5</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -10108,27 +10108,27 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Hyperparameter optimization</t>
+          <t>Dataset Recording Counts</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt</t>
+          <t>outputs/13_figures_diagrams/G01_dataset_recording_counts.png</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>src/evaluation/tuned.py; src/optimization/base.py; src/optimization/bayesian.py</t>
+          <t>outputs/13_figures_diagrams/G01_dataset_recording_counts.csv</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-07</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:11.262721+00:00</t>
+          <t>2026-08-30T10:48:42.372233+00:00</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -10138,19 +10138,19 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ALG-08</t>
+          <t>G02</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>O3</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -10158,27 +10158,27 @@
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>SVM training and probability calibration</t>
+          <t>Class Distribution</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.txt</t>
+          <t>outputs/13_figures_diagrams/G02_class_distribution.png</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>src/models/calibration.py; src/models/estimators.py</t>
+          <t>outputs/13_figures_diagrams/G02_class_distribution.csv</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-08</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:12.388722+00:00</t>
+          <t>2026-08-30T10:48:47.021026+00:00</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -10188,19 +10188,19 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ALG-09</t>
+          <t>G03</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>O3</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
@@ -10208,27 +10208,27 @@
       <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Random Forest training</t>
+          <t>Class Distribution Shares</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-09_random_forest_training.txt</t>
+          <t>outputs/13_figures_diagrams/G03_class_distribution_shares.png</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>src/feature_selection/ranking.py; src/models/estimators.py; src/models/pipeline.py</t>
+          <t>outputs/13_figures_diagrams/G03_class_distribution_shares.csv</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-09</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:12.492425+00:00</t>
+          <t>2026-08-30T10:48:49.860132+00:00</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -10238,19 +10238,19 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ALG-10</t>
+          <t>G04</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>O3</t>
+          <t>O1 (corpus definition)</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -10258,27 +10258,27 @@
       <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Gradient Boosting training</t>
+          <t>Recording Duration Histogram</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-10_gradient_boosting_training.txt</t>
+          <t>outputs/13_figures_diagrams/G04_recording_duration_histogram.png</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>src/models/estimators.py; src/models/weighting.py</t>
+          <t>outputs/13_figures_diagrams/G04_recording_duration_histogram.csv</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-10</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:12.613118+00:00</t>
+          <t>2026-08-30T10:48:54.156832+00:00</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -10288,47 +10288,51 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ALG-11</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>O3</t>
+          <t>O3 (preprocessing pipeline)</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
-      <c r="D189" t="inlineStr"/>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Equal-weight soft voting</t>
+          <t>Before And After Filtering</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-11_equal_weight_soft_voting.txt</t>
+          <t>outputs/13_figures_diagrams/G05_before_and_after_filtering.png</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>src/ensemble/soft_voting.py; src/models/estimators.py</t>
+          <t>outputs/13_figures_diagrams/G05_before_and_after_filtering.csv</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-11</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:12.806828+00:00</t>
+          <t>2026-08-30T10:48:57.234249+00:00</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -10338,47 +10342,51 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ALG-12</t>
+          <t>G06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>O3, O5</t>
+          <t>O3 (preprocessing pipeline)</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
-      <c r="D190" t="inlineStr"/>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Optimized-weight soft voting</t>
+          <t>Normal Versus Abnormal Spectrogram</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt</t>
+          <t>outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.png</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>src/ensemble/soft_voting.py</t>
+          <t>outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.csv</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-12</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:12.955723+00:00</t>
+          <t>2026-08-30T10:48:59.885736+00:00</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -10395,40 +10403,44 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ALG-13</t>
+          <t>G07</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
-      <c r="D191" t="inlineStr"/>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Binary evaluation workflow</t>
+          <t>MFCC Heatmap</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-13_binary_evaluation_workflow.txt</t>
+          <t>outputs/13_figures_diagrams/G07_mfcc_heatmap.png</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/evaluation/tuned.py</t>
+          <t>outputs/13_figures_diagrams/G07_mfcc_heatmap.csv</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-13</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.125306+00:00</t>
+          <t>2026-08-30T10:49:03.107896+00:00</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -10438,47 +10450,51 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ALG-14</t>
+          <t>G08</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>O6</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
-      <c r="D192" t="inlineStr"/>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Multiclass evaluation workflow</t>
+          <t>Chroma Heatmap</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.txt</t>
+          <t>outputs/13_figures_diagrams/G08_chroma_heatmap.png</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/reporting/multiclass_report.py</t>
+          <t>outputs/13_figures_diagrams/G08_chroma_heatmap.csv</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-14</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.256767+00:00</t>
+          <t>2026-08-30T10:49:04.751595+00:00</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -10488,47 +10504,51 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>ALG-15</t>
+          <t>G09</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>O1, O3</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
-      <c r="D193" t="inlineStr"/>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>CirCor subject-level aggregation</t>
+          <t>Wavelet Decomposition</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.txt</t>
+          <t>outputs/13_figures_diagrams/G09_wavelet_decomposition.png</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>src/evaluation/aggregation.py</t>
+          <t>outputs/13_figures_diagrams/G09_wavelet_decomposition.csv</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-15</t>
+          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.376578+00:00</t>
+          <t>2026-08-30T10:49:09.173960+00:00</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -10545,12 +10565,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ALG-16</t>
+          <t>FE-01</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
@@ -10558,27 +10578,27 @@
       <c r="E194" t="inlineStr"/>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Cross-dataset external validation</t>
+          <t>all 138 features with family, extractor, equation reference and unit</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-16_cross_dataset_external_validation.txt</t>
+          <t>outputs/03_features/feature_inventory.csv</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>scripts/13_finalize_binary_model.py; src/evaluation/transfer.py; src/models/registry.py</t>
+          <t>src/feature_extraction/registry.py</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-16</t>
+          <t>python -c "from src.feature_extraction.extractor import write_feature_artifacts; write_feature_artifacts()"</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.521701+00:00</t>
+          <t>2026-08-27T07:49:03.936944+00:00</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -10588,19 +10608,19 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ALG-17</t>
+          <t>FE-02</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
@@ -10608,27 +10628,27 @@
       <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Noise and duration robustness analysis</t>
+          <t>six feature families and their locked counts</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.txt</t>
+          <t>outputs/03_features/feature_family_summary.csv</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>scripts/23_noise_robustness.py; scripts/24_duration_robustness.py; src/evaluation/duration.py; src/evaluation/robustness.py</t>
+          <t>src/feature_extraction/registry.py</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-17</t>
+          <t>python -c "from src.feature_extraction.extractor import write_feature_artifacts; write_feature_artifacts()"</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.663479+00:00</t>
+          <t>2026-08-27T07:49:03.948244+00:00</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -10638,47 +10658,51 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ALG-18</t>
+          <t>FE-07</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>O1, O4</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
-      <c r="D196" t="inlineStr"/>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Failure case analysis</t>
+          <t>chroma heatmap, representative record</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-18_failure_case_analysis.txt</t>
+          <t>outputs/03_features/chroma_heatmap.png</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>src/evaluation/failure_analysis.py; src/reporting/failure_report.py</t>
+          <t>outputs/01_dataset_audit/metadata_master.csv</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-18</t>
+          <t>python -c "from src.feature_extraction.figures import generate_all; generate_all()"</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.807235+00:00</t>
+          <t>2026-08-27T07:14:10.687263+00:00</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -10688,47 +10712,51 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>ALG-19</t>
+          <t>FE-08</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>O1</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
-      <c r="D197" t="inlineStr"/>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Sample-level report generation</t>
+          <t>db4 multi-level decomposition, representative record</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-19_sample_level_report_generation.txt</t>
+          <t>outputs/03_features/wavelet_decomposition.png</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>src/feature_extraction/extractor.py; src/inference/predictor.py; src/preprocessing/pipeline.py; src/reporting/sample_report.py</t>
+          <t>outputs/01_dataset_audit/metadata_master.csv</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>python scripts/39_export_algorithms.py --ids ALG-19</t>
+          <t>python -c "from src.feature_extraction.figures import generate_all; generate_all()"</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>2026-09-11T13:04:13.956455+00:00</t>
+          <t>2026-08-27T07:14:12.086040+00:00</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -10738,47 +10766,51 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>FE-09</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
+          <t>O4 (feature engineering)</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
-      <c r="D198" t="inlineStr"/>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
       <c r="E198" t="inlineStr"/>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Dataset Inventory</t>
+          <t>amplitude envelope and detected peaks, representative record</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/T01_dataset_inventory.csv</t>
+          <t>outputs/03_features/signal_envelope.png</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/dataset_inventory.csv</t>
+          <t>outputs/01_dataset_audit/metadata_master.csv</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
+          <t>python -c "from src.feature_extraction.figures import generate_all; generate_all()"</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>2026-08-30T10:47:59.290988+00:00</t>
+          <t>2026-08-27T07:14:12.653769+00:00</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -10795,40 +10827,48 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>T02</t>
+          <t>MODEL-M1</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
-      <c r="D199" t="inlineStr"/>
-      <c r="E199" t="inlineStr"/>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Class Distribution and Imbalance Ratio</t>
+          <t>saved M1 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/T02_class_distribution_and_imbalance_ratio.csv</t>
+          <t>models_saved/binary/M1/manifest.json</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/class_distribution.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:00.613926+00:00</t>
+          <t>2026-08-28T11:52:03.259682+00:00</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -10845,40 +10885,48 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>T03</t>
+          <t>MODEL-M2</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
-      <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Recording Duration and Sampling Summary</t>
+          <t>saved M2 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/T03_recording_duration_and_sampling_summary.csv</t>
+          <t>models_saved/binary/M2/manifest.json</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/recording_duration_summary.csv; outputs/01_dataset_audit/sampling_rate_summary.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:01.979486+00:00</t>
+          <t>2026-08-28T11:52:03.814494+00:00</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -10888,47 +10936,55 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>MODEL-M3</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>O3 (preprocessing pipeline)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
-      <c r="D201" t="inlineStr"/>
-      <c r="E201" t="inlineStr"/>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Preprocessing Configuration</t>
+          <t>saved M3 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>outputs/02_preprocessing/T04_preprocessing_configuration.csv</t>
+          <t>models_saved/binary/M3/manifest.json</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>outputs/02_preprocessing/preprocessing_settings.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:03.098584+00:00</t>
+          <t>2026-08-28T11:52:04.537411+00:00</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -10945,40 +11001,48 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>MODEL-M4</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
-      <c r="D202" t="inlineStr"/>
-      <c r="E202" t="inlineStr"/>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Feature Inventory and Counts</t>
+          <t>saved M4 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>outputs/03_features/T05_feature_inventory_and_counts.csv</t>
+          <t>models_saved/binary/M4/manifest.json</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>outputs/03_features/feature_inventory.csv; outputs/03_features/feature_family_summary.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:04.059902+00:00</t>
+          <t>2026-08-28T11:52:13.812464+00:00</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -10988,47 +11052,55 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>T06</t>
+          <t>MODEL-M5</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>O5 (model configuration)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
-      <c r="D203" t="inlineStr"/>
-      <c r="E203" t="inlineStr"/>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Model Hyperparameter Configuration</t>
+          <t>saved M5 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>outputs/04_models/T06_model_hyperparameter_configuration.csv</t>
+          <t>models_saved/binary/M5/manifest.json</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>outputs/04_models/model_registry.csv; outputs/04_models/model_search_spaces.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>python scripts/18_setup_tables.py --tables T01 T02 T03 T04 T05 T06 T07</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:05.360215+00:00</t>
+          <t>2026-08-28T11:52:14.201923+00:00</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -11038,47 +11110,55 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>G01</t>
+          <t>MODEL-M6</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
-      <c r="D204" t="inlineStr"/>
-      <c r="E204" t="inlineStr"/>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Dataset Recording Counts</t>
+          <t>saved M6 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G01_dataset_recording_counts.png</t>
+          <t>models_saved/binary/M6/manifest.json</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G01_dataset_recording_counts.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:42.372233+00:00</t>
+          <t>2026-08-28T11:52:24.790974+00:00</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -11095,40 +11175,48 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>G02</t>
+          <t>MODEL-M7</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
-      <c r="D205" t="inlineStr"/>
-      <c r="E205" t="inlineStr"/>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Class Distribution</t>
+          <t>saved M7 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G02_class_distribution.png</t>
+          <t>models_saved/binary/M7/manifest.json</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G02_class_distribution.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:47.021026+00:00</t>
+          <t>2026-08-28T11:52:35.184798+00:00</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -11145,40 +11233,48 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>G03</t>
+          <t>MODEL-M8</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
+          <t>O3 (model training)</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
-      <c r="D206" t="inlineStr"/>
-      <c r="E206" t="inlineStr"/>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Class Distribution Shares</t>
+          <t>saved M8 (binary, fold 0 smoke fit): size, timing, features, versions</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G03_class_distribution_shares.png</t>
+          <t>models_saved/binary/M8/manifest.json</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G03_class_distribution_shares.csv</t>
+          <t>outputs/03_features/all_features_matrix.parquet</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/04_model_smoke.py</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:49.860132+00:00</t>
+          <t>2026-08-28T11:52:35.707776+00:00</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -11195,40 +11291,48 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>G04</t>
+          <t>EXP-F2-A9-DEFAULT</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>O1 (corpus definition)</t>
-        </is>
-      </c>
-      <c r="C207" t="inlineStr"/>
-      <c r="D207" t="inlineStr"/>
+          <t>O3 (optimization)</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>EXP-F2</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Recording Duration Histogram</t>
+          <t>A9 best individual model vs ensemble, default parameters</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G04_recording_duration_histogram.png</t>
+          <t>outputs/09_ablation/A9_individual_vs_ensemble_default.csv</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G04_recording_duration_histogram.csv</t>
+          <t>outputs/09_ablation/optimization_ablation_per_fold.csv</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/27_optimization_ablation.py</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:54.156832+00:00</t>
+          <t>2026-09-11T05:48:21.643279+00:00</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -11245,44 +11349,48 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>EXP-F2-A9-TUNED</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>O3 (preprocessing pipeline)</t>
-        </is>
-      </c>
-      <c r="C208" t="inlineStr"/>
+          <t>O3 (optimization)</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>EXP-F2</t>
+        </is>
+      </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1 PhysioNet 2016</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Before And After Filtering</t>
+          <t>A9 best individual model vs ensemble, tuned parameters</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G05_before_and_after_filtering.png</t>
+          <t>outputs/09_ablation/A9_individual_vs_ensemble_tuned.csv</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G05_before_and_after_filtering.csv</t>
+          <t>outputs/09_ablation/optimization_ablation_per_fold.csv</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/27_optimization_ablation.py</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:57.234249+00:00</t>
+          <t>2026-09-11T05:48:21.636175+00:00</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -11299,44 +11407,48 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>G06</t>
+          <t>EXP-F2-A10</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>O3 (preprocessing pipeline)</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr"/>
+          <t>O3 (optimization)</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>EXP-F2</t>
+        </is>
+      </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1 PhysioNet 2016</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Normal Versus Abnormal Spectrogram</t>
+          <t>A10 equal-weight vs optimized-weight ensemble</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.png</t>
+          <t>outputs/09_ablation/A10_equal_vs_optimized_weights.csv</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G06_normal_versus_abnormal_spectrogram.csv</t>
+          <t>outputs/09_ablation/optimization_ablation_per_fold.csv</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/27_optimization_ablation.py</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>2026-08-30T10:48:59.885736+00:00</t>
+          <t>2026-09-11T05:48:21.644289+00:00</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -11353,44 +11465,48 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>G07</t>
+          <t>STAT-BOOTSTRAP</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr"/>
+          <t>O3 (model comparison)</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>EXP-A1, EXP-A2</t>
+        </is>
+      </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1 PhysioNet 2016</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
         <is>
-          <t>MFCC Heatmap</t>
+          <t>bootstrap ROC-AUC confidence intervals, key binary results</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G07_mfcc_heatmap.png</t>
+          <t>outputs/12_statistics/bootstrap_auc_ci.csv</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G07_mfcc_heatmap.csv</t>
+          <t>outputs/06_binary_results/EXP-A1/predictions.parquet; outputs/06_binary_results/EXP-A2/predictions.parquet; outputs/07_multiclass_results/EXP-B1/predictions.parquet; outputs/07_multiclass_results/EXP-B2/predictions.parquet; outputs/08_circor_external_validation/EXP-C1-three_class/predictions.parquet; outputs/08_circor_external_validation/EXP-C1-two_class/predictions.parquet; outputs/08_circor_external_validation/EXP-C2/predictions.parquet</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/34_statistical_validation.py</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>2026-08-30T10:49:03.107896+00:00</t>
+          <t>2026-09-10T12:50:09.228259+00:00</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -11400,51 +11516,51 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 7 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>Q1_T01</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
+          <t>O1, O6</t>
         </is>
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1-D4</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Chroma Heatmap</t>
+          <t>Dataset Summary</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G08_chroma_heatmap.png</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T01_dataset_summary.csv</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G08_chroma_heatmap.csv</t>
+          <t>outputs/01_dataset_audit/T01_dataset_inventory.csv</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>2026-08-30T10:49:04.751595+00:00</t>
+          <t>2026-09-11T14:19:00.716235+00:00</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -11461,44 +11577,40 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>G09</t>
+          <t>Q1_T02</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
+          <t>O4</t>
         </is>
       </c>
       <c r="C212" t="inlineStr"/>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
+      <c r="D212" t="inlineStr"/>
       <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Wavelet Decomposition</t>
+          <t>Feature Summary</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G09_wavelet_decomposition.png</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T02_feature_summary.csv</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/G09_wavelet_decomposition.csv</t>
+          <t>outputs/03_features/T05_feature_inventory_and_counts.csv</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>python scripts/19_data_graphs.py --figures G01 G02 G03 G04 G05 G06 G07 G08 G09 G10</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>2026-08-30T10:49:09.173960+00:00</t>
+          <t>2026-09-11T14:19:00.941107+00:00</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -11515,40 +11627,48 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>FE-01</t>
+          <t>Q1_T03</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>SO-01, SO-02</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
         <is>
-          <t>all 138 features with family, extractor, equation reference and unit</t>
+          <t>Model and Search Configuration</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>outputs/03_features/feature_inventory.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T03_model_and_search_configuration.csv</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>src/feature_extraction/registry.py</t>
+          <t>outputs/05_search_optimization/T07_search_space_and_best_parameters.csv</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>python -c "from src.feature_extraction.extractor import write_feature_artifacts; write_feature_artifacts()"</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>2026-08-27T07:49:03.936944+00:00</t>
+          <t>2026-09-11T14:19:01.282609+00:00</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -11565,40 +11685,48 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>FE-02</t>
+          <t>Q1_T04</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr"/>
-      <c r="D214" t="inlineStr"/>
+          <t>O1, O3</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>EXP-A2</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>D1 PhysioNet 2016</t>
+        </is>
+      </c>
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
-          <t>six feature families and their locked counts</t>
+          <t>Individual versus Ensemble</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>outputs/03_features/feature_family_summary.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T04_individual_versus_ensemble.csv</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>src/feature_extraction/registry.py</t>
+          <t>outputs/06_binary_results/T08_physionet_individual_model_comparison.csv</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>python -c "from src.feature_extraction.extractor import write_feature_artifacts; write_feature_artifacts()"</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>2026-08-27T07:49:03.948244+00:00</t>
+          <t>2026-09-11T14:19:01.548872+00:00</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -11615,44 +11743,48 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>FE-07</t>
+          <t>Q1_T05</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr"/>
+          <t>O2, O5</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>EXP-F1</t>
+        </is>
+      </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1 PhysioNet 2016</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
         <is>
-          <t>chroma heatmap, representative record</t>
+          <t>Feature Ablation</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>outputs/03_features/chroma_heatmap.png</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T05_feature_ablation.csv</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/metadata_master.csv</t>
+          <t>outputs/09_ablation/T17_feature_family_ablation.csv</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>python -c "from src.feature_extraction.figures import generate_all; generate_all()"</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>2026-08-27T07:14:10.687263+00:00</t>
+          <t>2026-09-11T14:19:01.840856+00:00</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -11669,44 +11801,48 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>FE-08</t>
+          <t>Q1_T06</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr"/>
+          <t>O3, O5</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>EXP-F2</t>
+        </is>
+      </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1 PhysioNet 2016</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
-          <t>db4 multi-level decomposition, representative record</t>
+          <t>Optimization Ablation</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>outputs/03_features/wavelet_decomposition.png</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T06_optimization_ablation.csv</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/metadata_master.csv</t>
+          <t>outputs/09_ablation/T19_search_and_optimization_ablation.csv</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>python -c "from src.feature_extraction.figures import generate_all; generate_all()"</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>2026-08-27T07:14:12.086040+00:00</t>
+          <t>2026-09-11T14:19:02.104372+00:00</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -11723,44 +11859,48 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>FE-09</t>
+          <t>Q1_T07</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>O4 (feature engineering)</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr"/>
+          <t>O6</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>EXP-B1, EXP-B2</t>
+        </is>
+      </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2 PASCAL A; D3 PASCAL B</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
-          <t>amplitude envelope and detected peaks, representative record</t>
+          <t>Multiclass Results</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>outputs/03_features/signal_envelope.png</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T07_multiclass_results.csv</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/metadata_master.csv</t>
+          <t>outputs/07_multiclass_results/T11_pascal_a_multiclass_results.csv; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.csv</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>python -c "from src.feature_extraction.figures import generate_all; generate_all()"</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>2026-08-27T07:14:12.653769+00:00</t>
+          <t>2026-09-11T14:19:02.418832+00:00</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -11770,55 +11910,55 @@
       </c>
       <c r="L217" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>MODEL-M1</t>
+          <t>Q1_T08</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr"/>
+          <t>O1, O3, O6</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>EXP-C1, EXP-C2, EXP-D1, EXP-F3</t>
+        </is>
+      </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
+          <t>D4 CirCor 2022; D1 PhysioNet 2016</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
-          <t>saved M1 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>External Validation</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>models_saved/binary/M1/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T08_external_validation.csv</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/08_circor_external_validation/T13_circor_murmur_classification_results.csv; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.csv; outputs/08_circor_external_validation/T16_cross_dataset_generalization.csv; outputs/09_ablation/T-S5_leave_one_source_out_generalization.csv</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:03.259682+00:00</t>
+          <t>2026-09-11T14:19:02.861569+00:00</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -11828,55 +11968,55 @@
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>MODEL-M2</t>
+          <t>Q1_T09</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr"/>
+          <t>O4, O5</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>EXP-A2, EXP-E1, EXP-E2</t>
+        </is>
+      </c>
       <c r="D219" t="inlineStr">
         <is>
           <t>D1 PhysioNet 2016</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
+      <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>saved M2 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>Complexity and Robustness</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>models_saved/binary/M2/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_T09_complexity_and_robustness.csv</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/11_complexity/T24_complexity_analysis.csv; outputs/09_robustness_analysis/T20_noise_robustness.csv; outputs/09_robustness_analysis/T21_duration_robustness.csv</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:03.814494+00:00</t>
+          <t>2026-09-11T14:19:03.218971+00:00</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -11886,55 +12026,55 @@
       </c>
       <c r="L219" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>MODEL-M3</t>
+          <t>Q1_G01</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr"/>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>EXP-A2</t>
+        </is>
+      </c>
       <c r="D220" t="inlineStr">
         <is>
           <t>D1 PhysioNet 2016</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
+      <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
-          <t>saved M3 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>ROC and PR Combined</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>models_saved/binary/M3/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G01_roc_and_pr_combined.png</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G01_roc_and_pr_combined.csv</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:04.537411+00:00</t>
+          <t>2026-09-11T14:19:05.421649+00:00</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -11951,48 +12091,48 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>MODEL-M4</t>
+          <t>Q1_G02</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr"/>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>EXP-A2</t>
+        </is>
+      </c>
       <c r="D221" t="inlineStr">
         <is>
           <t>D1 PhysioNet 2016</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
+      <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
-          <t>saved M4 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>Binary Confusion Matrix</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>models_saved/binary/M4/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G02_binary_confusion_matrix.png</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G02_binary_confusion_matrix.csv</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:13.812464+00:00</t>
+          <t>2026-09-11T14:19:05.852433+00:00</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -12009,48 +12149,48 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MODEL-M5</t>
+          <t>Q1_G03</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr"/>
+          <t>O6</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>EXP-B1, EXP-B2</t>
+        </is>
+      </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
+          <t>D2 PASCAL A; D3 PASCAL B</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
-          <t>saved M5 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>Multiclass Confusion Matrix</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>models_saved/binary/M5/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G03_multiclass_confusion_matrix.png</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G03_multiclass_confusion_matrix.csv</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:14.201923+00:00</t>
+          <t>2026-09-11T14:19:06.885769+00:00</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -12067,48 +12207,48 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MODEL-M6</t>
+          <t>Q1_G04</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr"/>
+          <t>O3, O5</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>EXP-F1, EXP-F2</t>
+        </is>
+      </c>
       <c r="D223" t="inlineStr">
         <is>
           <t>D1 PhysioNet 2016</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>M6</t>
-        </is>
-      </c>
+      <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
-          <t>saved M6 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>Ablation and Optimization</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>models_saved/binary/M6/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G04_ablation_and_optimization.png</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G04_ablation_and_optimization.csv</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:24.790974+00:00</t>
+          <t>2026-09-11T14:19:07.903782+00:00</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -12125,48 +12265,48 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>MODEL-M7</t>
+          <t>Q1_G05</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr"/>
+          <t>O1, O5</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>EXP-A2, EXP-D1</t>
+        </is>
+      </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>M7</t>
-        </is>
-      </c>
+          <t>D1 PhysioNet 2016; D4 CirCor 2022</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
-          <t>saved M7 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>Generalization and Complexity</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>models_saved/binary/M7/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G05_generalization_and_complexity.png</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_G05_generalization_and_complexity.csv</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:35.184798+00:00</t>
+          <t>2026-09-11T14:19:09.412080+00:00</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -12183,48 +12323,40 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>MODEL-M8</t>
+          <t>Q1_F01</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>O3 (model training)</t>
+          <t>O1, O3</t>
         </is>
       </c>
       <c r="C225" t="inlineStr"/>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>M8</t>
-        </is>
-      </c>
+      <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
-          <t>saved M8 (binary, fold 0 smoke fit): size, timing, features, versions</t>
+          <t>proposed architecture</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>models_saved/binary/M8/manifest.json</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_F01_proposed_architecture.png</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>outputs/03_features/all_features_matrix.parquet</t>
+          <t>outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.svg</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>python scripts/04_model_smoke.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>2026-08-28T11:52:35.707776+00:00</t>
+          <t>2026-09-11T14:19:09.435611+00:00</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -12241,48 +12373,40 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>EXP-F2-A9-DEFAULT</t>
+          <t>Q1_F02</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>O3 (optimization)</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>EXP-F2</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O1, O3</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr"/>
+      <c r="D226" t="inlineStr"/>
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
-          <t>A9 best individual model vs ensemble, default parameters</t>
+          <t>feature and ensemble workflow</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/A9_individual_vs_ensemble_default.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_F02_feature_and_ensemble_workflow.png</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/optimization_ablation_per_fold.csv</t>
+          <t>outputs/13_figures_diagrams/F08_feature_family_fusion.svg; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.svg</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>python scripts/27_optimization_ablation.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>2026-09-11T05:48:21.643279+00:00</t>
+          <t>2026-09-11T14:19:09.900031+00:00</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -12292,55 +12416,47 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>EXP-F2-A9-TUNED</t>
+          <t>Q1_ALG01</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>O3 (optimization)</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>EXP-F2</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O3, O4, O5</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr"/>
+      <c r="D227" t="inlineStr"/>
       <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
-          <t>A9 best individual model vs ensemble, tuned parameters</t>
+          <t>ALG-04 as feature extraction</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/A9_individual_vs_ensemble_tuned.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_ALG01_feature_extraction.docx</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/optimization_ablation_per_fold.csv</t>
+          <t>outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>python scripts/27_optimization_ablation.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>2026-09-11T05:48:21.636175+00:00</t>
+          <t>2026-09-11T14:19:09.931267+00:00</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -12357,48 +12473,40 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>EXP-F2-A10</t>
+          <t>Q1_ALG02</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>O3 (optimization)</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>EXP-F2</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O3, O4, O5</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr"/>
+      <c r="D228" t="inlineStr"/>
       <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
         <is>
-          <t>A10 equal-weight vs optimized-weight ensemble</t>
+          <t>ALG-07 as search optimization</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/A10_equal_vs_optimized_weights.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_ALG02_search_optimization.docx</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/optimization_ablation_per_fold.csv</t>
+          <t>outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>python scripts/27_optimization_ablation.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>2026-09-11T05:48:21.644289+00:00</t>
+          <t>2026-09-11T14:19:09.948493+00:00</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -12415,48 +12523,40 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>STAT-BOOTSTRAP</t>
+          <t>Q1_ALG03</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>O3 (model comparison)</t>
-        </is>
-      </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>EXP-A1, EXP-A2</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O3, O4, O5</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr"/>
+      <c r="D229" t="inlineStr"/>
       <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
-          <t>bootstrap ROC-AUC confidence intervals, key binary results</t>
+          <t>ALG-12 as proposed ensemble</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>outputs/12_statistics/bootstrap_auc_ci.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_ALG03_proposed_ensemble.docx</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>outputs/06_binary_results/EXP-A1/predictions.parquet; outputs/06_binary_results/EXP-A2/predictions.parquet; outputs/07_multiclass_results/EXP-B1/predictions.parquet; outputs/07_multiclass_results/EXP-B2/predictions.parquet; outputs/08_circor_external_validation/EXP-C1-three_class/predictions.parquet; outputs/08_circor_external_validation/EXP-C1-two_class/predictions.parquet; outputs/08_circor_external_validation/EXP-C2/predictions.parquet</t>
+          <t>outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>python scripts/34_statistical_validation.py</t>
+          <t>python scripts/43_q1_assets.py</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>2026-09-10T12:50:09.228259+00:00</t>
+          <t>2026-09-11T14:19:09.982718+00:00</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -12466,41 +12566,37 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>file and 7 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Q1_T01</t>
+          <t>Q1_NARRATIVE</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>O1, O6</t>
+          <t>O1-O6</t>
         </is>
       </c>
       <c r="C230" t="inlineStr"/>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>D1-D4</t>
-        </is>
-      </c>
+      <c r="D230" t="inlineStr"/>
       <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Dataset Summary</t>
+          <t>results narrative written from generated numbers</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T01_dataset_summary.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_results_narrative.docx</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>outputs/01_dataset_audit/T01_dataset_inventory.csv</t>
+          <t>outputs/Q1_PAPER_ASSETS/Q1_results_narrative_sources.csv</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -12510,7 +12606,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:00.716235+00:00</t>
+          <t>2026-09-11T14:19:10.990835+00:00</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -12527,12 +12623,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Q1_T02</t>
+          <t>ALG-01</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>O4</t>
+          <t>O1, O6</t>
         </is>
       </c>
       <c r="C231" t="inlineStr"/>
@@ -12540,27 +12636,27 @@
       <c r="E231" t="inlineStr"/>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Feature Summary</t>
+          <t>Dataset loading and master metadata construction</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T02_feature_summary.csv</t>
+          <t>outputs/14_algorithms/ALG-01_dataset_loading_and_master_metadata_construction.txt</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>outputs/03_features/T05_feature_inventory_and_counts.csv</t>
+          <t>src/data_loader/catalog.py; src/data_loader/circor.py; src/data_loader/duplicates.py; src/data_loader/integrity.py; src/data_loader/master.py; src/data_loader/pascal.py; src/data_loader/physionet.py</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-01</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:00.941107+00:00</t>
+          <t>2026-09-11T14:51:05.934979+00:00</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -12570,55 +12666,47 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 7 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Q1_T03</t>
+          <t>ALG-02</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>O5</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>SO-01, SO-02</t>
-        </is>
-      </c>
-      <c r="D232" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O4</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr"/>
+      <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Model and Search Configuration</t>
+          <t>Signal harmonization and resampling</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T03_model_and_search_configuration.csv</t>
+          <t>outputs/14_algorithms/ALG-02_signal_harmonization_and_resampling.txt</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>outputs/05_search_optimization/T07_search_space_and_best_parameters.csv</t>
+          <t>src/preprocessing/io.py; src/preprocessing/pipeline.py; src/preprocessing/quality.py</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-02</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:01.282609+00:00</t>
+          <t>2026-09-11T14:51:06.211098+00:00</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -12628,55 +12716,47 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Q1_T04</t>
+          <t>ALG-03</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>O1, O3</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>EXP-A2</t>
-        </is>
-      </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O4</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr"/>
+      <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Individual versus Ensemble</t>
+          <t>Butterworth filtering and z-score normalization</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T04_individual_versus_ensemble.csv</t>
+          <t>outputs/14_algorithms/ALG-03_butterworth_filtering_and_z_score_normalization.txt</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>outputs/06_binary_results/T08_physionet_individual_model_comparison.csv</t>
+          <t>src/preprocessing/filters.py; src/preprocessing/normalize.py</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-03</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:01.548872+00:00</t>
+          <t>2026-09-11T14:51:08.176513+00:00</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -12686,55 +12766,47 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Q1_T05</t>
+          <t>ALG-04</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>O2, O5</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>EXP-F1</t>
-        </is>
-      </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O4</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr"/>
+      <c r="D234" t="inlineStr"/>
       <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Feature Ablation</t>
+          <t>Multi-domain 138-feature extraction</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T05_feature_ablation.csv</t>
+          <t>outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/T17_feature_family_ablation.csv</t>
+          <t>src/feature_extraction/extractor.py; src/feature_extraction/registry.py</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-04</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:01.840856+00:00</t>
+          <t>2026-09-11T14:51:08.297525+00:00</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -12744,55 +12816,47 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Q1_T06</t>
+          <t>ALG-05</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>O3, O5</t>
-        </is>
-      </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>EXP-F2</t>
-        </is>
-      </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr"/>
+      <c r="D235" t="inlineStr"/>
       <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Optimization Ablation</t>
+          <t>Fold-safe scaling and preprocessing</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T06_optimization_ablation.csv</t>
+          <t>outputs/14_algorithms/ALG-05_fold_safe_scaling_and_preprocessing.txt</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>outputs/09_ablation/T19_search_and_optimization_ablation.csv</t>
+          <t>src/data_loader/splits.py; src/models/pipeline.py</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-05</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:02.104372+00:00</t>
+          <t>2026-09-11T14:51:08.429879+00:00</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -12802,55 +12866,47 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Q1_T07</t>
+          <t>ALG-06</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>O6</t>
-        </is>
-      </c>
-      <c r="C236" t="inlineStr">
-        <is>
-          <t>EXP-B1, EXP-B2</t>
-        </is>
-      </c>
-      <c r="D236" t="inlineStr">
-        <is>
-          <t>D2 PASCAL A; D3 PASCAL B</t>
-        </is>
-      </c>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr"/>
+      <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Multiclass Results</t>
+          <t>Search based feature selection</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T07_multiclass_results.csv</t>
+          <t>outputs/14_algorithms/ALG-06_search_based_feature_selection.txt</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>outputs/07_multiclass_results/T11_pascal_a_multiclass_results.csv; outputs/07_multiclass_results/T12_pascal_b_multiclass_results.csv</t>
+          <t>src/feature_selection/ranking.py; src/feature_selection/sweep.py; src/optimization/base.py; src/optimization/multi_objective.py</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-06</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:02.418832+00:00</t>
+          <t>2026-09-11T14:51:08.598593+00:00</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -12860,55 +12916,47 @@
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Q1_T08</t>
+          <t>ALG-07</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>O1, O3, O6</t>
-        </is>
-      </c>
-      <c r="C237" t="inlineStr">
-        <is>
-          <t>EXP-C1, EXP-C2, EXP-D1, EXP-F3</t>
-        </is>
-      </c>
-      <c r="D237" t="inlineStr">
-        <is>
-          <t>D4 CirCor 2022; D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr"/>
+      <c r="D237" t="inlineStr"/>
       <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
-          <t>External Validation</t>
+          <t>Hyperparameter optimization</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T08_external_validation.csv</t>
+          <t>outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>outputs/08_circor_external_validation/T13_circor_murmur_classification_results.csv; outputs/08_circor_external_validation/T14_circor_clinical_outcome_results.csv; outputs/08_circor_external_validation/T16_cross_dataset_generalization.csv; outputs/09_ablation/T-S5_leave_one_source_out_generalization.csv</t>
+          <t>src/evaluation/tuned.py; src/optimization/base.py; src/optimization/bayesian.py</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-07</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:02.861569+00:00</t>
+          <t>2026-09-11T14:51:08.748632+00:00</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -12918,55 +12966,47 @@
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t>file and 4 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Q1_T09</t>
+          <t>ALG-08</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>O4, O5</t>
-        </is>
-      </c>
-      <c r="C238" t="inlineStr">
-        <is>
-          <t>EXP-A2, EXP-E1, EXP-E2</t>
-        </is>
-      </c>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr"/>
+      <c r="D238" t="inlineStr"/>
       <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Complexity and Robustness</t>
+          <t>SVM training and probability calibration</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_T09_complexity_and_robustness.csv</t>
+          <t>outputs/14_algorithms/ALG-08_svm_training_and_probability_calibration.txt</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>outputs/11_complexity/T24_complexity_analysis.csv; outputs/09_robustness_analysis/T20_noise_robustness.csv; outputs/09_robustness_analysis/T21_duration_robustness.csv</t>
+          <t>src/models/calibration.py; src/models/estimators.py</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-08</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:03.218971+00:00</t>
+          <t>2026-09-11T14:51:09.960299+00:00</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -12976,55 +13016,47 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t>file and 3 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Q1_G01</t>
+          <t>ALG-09</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="C239" t="inlineStr">
-        <is>
-          <t>EXP-A2</t>
-        </is>
-      </c>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr"/>
+      <c r="D239" t="inlineStr"/>
       <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
-          <t>ROC and PR Combined</t>
+          <t>Random Forest training</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G01_roc_and_pr_combined.png</t>
+          <t>outputs/14_algorithms/ALG-09_random_forest_training.txt</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G01_roc_and_pr_combined.csv</t>
+          <t>src/feature_selection/ranking.py; src/models/estimators.py; src/models/pipeline.py</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-09</t>
         </is>
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:05.421649+00:00</t>
+          <t>2026-09-11T14:51:10.075103+00:00</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -13034,55 +13066,47 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Q1_G02</t>
+          <t>ALG-10</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>O1</t>
-        </is>
-      </c>
-      <c r="C240" t="inlineStr">
-        <is>
-          <t>EXP-A2</t>
-        </is>
-      </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr"/>
+      <c r="D240" t="inlineStr"/>
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Binary Confusion Matrix</t>
+          <t>Gradient Boosting training</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G02_binary_confusion_matrix.png</t>
+          <t>outputs/14_algorithms/ALG-10_gradient_boosting_training.txt</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G02_binary_confusion_matrix.csv</t>
+          <t>src/models/estimators.py; src/models/weighting.py</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-10</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:05.852433+00:00</t>
+          <t>2026-09-11T14:51:10.202978+00:00</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -13092,55 +13116,47 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Q1_G03</t>
+          <t>ALG-11</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>O6</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>EXP-B1, EXP-B2</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>D2 PASCAL A; D3 PASCAL B</t>
-        </is>
-      </c>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr"/>
+      <c r="D241" t="inlineStr"/>
       <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Multiclass Confusion Matrix</t>
+          <t>Equal-weight soft voting</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G03_multiclass_confusion_matrix.png</t>
+          <t>outputs/14_algorithms/ALG-11_equal_weight_soft_voting.txt</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G03_multiclass_confusion_matrix.csv</t>
+          <t>src/ensemble/soft_voting.py; src/models/estimators.py</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-11</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:06.885769+00:00</t>
+          <t>2026-09-11T14:51:10.350065+00:00</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -13150,14 +13166,14 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Q1_G04</t>
+          <t>ALG-12</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -13165,40 +13181,32 @@
           <t>O3, O5</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>EXP-F1, EXP-F2</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016</t>
-        </is>
-      </c>
+      <c r="C242" t="inlineStr"/>
+      <c r="D242" t="inlineStr"/>
       <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Ablation and Optimization</t>
+          <t>Optimized-weight soft voting</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G04_ablation_and_optimization.png</t>
+          <t>outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G04_ablation_and_optimization.csv</t>
+          <t>src/ensemble/soft_voting.py</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-12</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:07.903782+00:00</t>
+          <t>2026-09-11T14:51:10.484315+00:00</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -13215,48 +13223,40 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Q1_G05</t>
+          <t>ALG-13</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>O1, O5</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>EXP-A2, EXP-D1</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>D1 PhysioNet 2016; D4 CirCor 2022</t>
-        </is>
-      </c>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr"/>
+      <c r="D243" t="inlineStr"/>
       <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Generalization and Complexity</t>
+          <t>Binary evaluation workflow</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G05_generalization_and_complexity.png</t>
+          <t>outputs/14_algorithms/ALG-13_binary_evaluation_workflow.txt</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_G05_generalization_and_complexity.csv</t>
+          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/evaluation/tuned.py</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-13</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:09.412080+00:00</t>
+          <t>2026-09-11T14:51:10.659834+00:00</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -13266,19 +13266,19 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Q1_F01</t>
+          <t>ALG-14</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>O1, O3</t>
+          <t>O6</t>
         </is>
       </c>
       <c r="C244" t="inlineStr"/>
@@ -13286,27 +13286,27 @@
       <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
-          <t>proposed architecture</t>
+          <t>Multiclass evaluation workflow</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_F01_proposed_architecture.png</t>
+          <t>outputs/14_algorithms/ALG-14_multiclass_evaluation_workflow.txt</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/F01_overall_pv_mepcg_proposed_architecture.svg</t>
+          <t>src/evaluation/cv.py; src/evaluation/experiment.py; src/evaluation/metrics.py; src/reporting/multiclass_report.py</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-14</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:09.435611+00:00</t>
+          <t>2026-09-11T14:51:10.824189+00:00</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -13316,14 +13316,14 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Q1_F02</t>
+          <t>ALG-15</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -13336,27 +13336,27 @@
       <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
-          <t>feature and ensemble workflow</t>
+          <t>CirCor subject-level aggregation</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_F02_feature_and_ensemble_workflow.png</t>
+          <t>outputs/14_algorithms/ALG-15_circor_subject_level_aggregation.txt</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>outputs/13_figures_diagrams/F08_feature_family_fusion.svg; outputs/13_figures_diagrams/F10_svm_rf_gb_optimized_soft_voting_architecture.svg</t>
+          <t>src/evaluation/aggregation.py</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-15</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:09.900031+00:00</t>
+          <t>2026-09-11T14:51:11.073258+00:00</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -13366,19 +13366,19 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t>file and 2 source path(s) on disk</t>
+          <t>file and 1 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Q1_ALG01</t>
+          <t>ALG-16</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>O3, O4, O5</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -13386,27 +13386,27 @@
       <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
-          <t>ALG-04 as feature extraction</t>
+          <t>Cross-dataset external validation</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_ALG01_feature_extraction.docx</t>
+          <t>outputs/14_algorithms/ALG-16_cross_dataset_external_validation.txt</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-04_multi_domain_138_feature_extraction.txt</t>
+          <t>scripts/13_finalize_binary_model.py; src/evaluation/transfer.py; src/models/registry.py</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-16</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:09.931267+00:00</t>
+          <t>2026-09-11T14:51:11.277367+00:00</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -13416,19 +13416,19 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 3 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Q1_ALG02</t>
+          <t>ALG-17</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>O3, O4, O5</t>
+          <t>O4</t>
         </is>
       </c>
       <c r="C247" t="inlineStr"/>
@@ -13436,27 +13436,27 @@
       <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
-          <t>ALG-07 as search optimization</t>
+          <t>Noise and duration robustness analysis</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_ALG02_search_optimization.docx</t>
+          <t>outputs/14_algorithms/ALG-17_noise_and_duration_robustness_analysis.txt</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-07_hyperparameter_optimization.txt</t>
+          <t>scripts/23_noise_robustness.py; scripts/24_duration_robustness.py; src/evaluation/duration.py; src/evaluation/robustness.py</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-17</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:09.948493+00:00</t>
+          <t>2026-09-11T14:51:11.438896+00:00</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -13466,19 +13466,19 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Q1_ALG03</t>
+          <t>ALG-18</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>O3, O4, O5</t>
+          <t>O1, O4</t>
         </is>
       </c>
       <c r="C248" t="inlineStr"/>
@@ -13486,27 +13486,27 @@
       <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
         <is>
-          <t>ALG-12 as proposed ensemble</t>
+          <t>Failure case analysis</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_ALG03_proposed_ensemble.docx</t>
+          <t>outputs/14_algorithms/ALG-18_failure_case_analysis.txt</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>outputs/14_algorithms/ALG-12_optimized_weight_soft_voting.txt</t>
+          <t>src/evaluation/failure_analysis.py; src/reporting/failure_report.py</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-18</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:09.982718+00:00</t>
+          <t>2026-09-11T14:51:11.583309+00:00</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -13516,19 +13516,19 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 2 source path(s) on disk</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Q1_NARRATIVE</t>
+          <t>ALG-19</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>O1-O6</t>
+          <t>O1</t>
         </is>
       </c>
       <c r="C249" t="inlineStr"/>
@@ -13536,27 +13536,27 @@
       <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
-          <t>results narrative written from generated numbers</t>
+          <t>Sample-level report generation</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_results_narrative.docx</t>
+          <t>outputs/14_algorithms/ALG-19_sample_level_report_generation.txt</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>outputs/Q1_PAPER_ASSETS/Q1_results_narrative_sources.csv</t>
+          <t>src/feature_extraction/extractor.py; src/inference/predictor.py; src/preprocessing/pipeline.py; src/reporting/sample_report.py</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>python scripts/43_q1_assets.py</t>
+          <t>python scripts/39_export_algorithms.py --ids ALG-19</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:10.990835+00:00</t>
+          <t>2026-09-11T14:51:11.739933+00:00</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -13566,7 +13566,7 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t>file and 1 source path(s) on disk</t>
+          <t>file and 4 source path(s) on disk</t>
         </is>
       </c>
     </row>
@@ -13614,7 +13614,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:22.283869+00:00</t>
+          <t>2026-09-11T14:54:04.488902+00:00</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -13672,7 +13672,7 @@
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:22.556059+00:00</t>
+          <t>2026-09-11T14:54:04.771116+00:00</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -13722,7 +13722,7 @@
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:24.068115+00:00</t>
+          <t>2026-09-11T14:54:06.283918+00:00</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -13772,7 +13772,7 @@
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:24.080120+00:00</t>
+          <t>2026-09-11T14:54:06.304806+00:00</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -13822,7 +13822,7 @@
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:24.089262+00:00</t>
+          <t>2026-09-11T14:54:06.327597+00:00</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -13880,7 +13880,7 @@
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:26.934308+00:00</t>
+          <t>2026-09-11T14:54:08.931213+00:00</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:27.204736+00:00</t>
+          <t>2026-09-11T14:54:09.222822+00:00</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -13988,7 +13988,7 @@
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:28.721129+00:00</t>
+          <t>2026-09-11T14:54:10.686688+00:00</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -14046,7 +14046,7 @@
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:37.763303+00:00</t>
+          <t>2026-09-11T14:54:19.717030+00:00</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -14104,7 +14104,7 @@
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:37.800597+00:00</t>
+          <t>2026-09-11T14:54:19.752713+00:00</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -14162,7 +14162,7 @@
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:37.824312+00:00</t>
+          <t>2026-09-11T14:54:19.781422+00:00</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -14220,7 +14220,7 @@
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:37.850786+00:00</t>
+          <t>2026-09-11T14:54:19.805267+00:00</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>2026-09-11T14:19:37.875177+00:00</t>
+          <t>2026-09-11T14:54:19.828051+00:00</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -14328,7 +14328,7 @@
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.088053+00:00</t>
+          <t>2026-09-11T14:54:45.716152+00:00</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -14378,7 +14378,7 @@
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.103675+00:00</t>
+          <t>2026-09-11T14:54:45.733006+00:00</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.156844+00:00</t>
+          <t>2026-09-11T14:54:45.771865+00:00</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -14478,7 +14478,7 @@
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.193039+00:00</t>
+          <t>2026-09-11T14:54:45.819255+00:00</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -14528,7 +14528,7 @@
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.280312+00:00</t>
+          <t>2026-09-11T14:54:45.891637+00:00</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -14578,7 +14578,7 @@
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.310953+00:00</t>
+          <t>2026-09-11T14:54:45.914467+00:00</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:10.344214+00:00</t>
+          <t>2026-09-11T14:54:45.948660+00:00</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11T14:24:13.539186+00:00</t>
+          <t>2026-09-11T14:54:48.156813+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>